<commit_message>
hvac-designer: handle real traced multi-plan sheets; add DDA housing worked example
Reader: several plans per sheet split by title, glyph-outline-on-ink label
voting, cell-type window schedules, decimal-metre dimension strings,
courtyards/shafts treated as exterior, title-block/grid noise dropped,
polyline door arcs, area tolerance for traced drawings, window-size and
conditioned overrides from project.json, fill_from_floor helper for
typical flats. Equipment: per-system outdoor unit location (facade/roof),
one ducted unit per room option, roof outline fallback, DS-18 size.
DXF background simplified on heavy drawings. Second worked example:
4-storey DDA MIG housing block (16 flats) run end to end.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WkbbzwcKHZubjtebdHFNYk
</commit_message>
<xml_diff>
--- a/.claude/skills/hvac-designer/examples/riyadh_villa/output/out/HVAC_BOQ.xlsx
+++ b/.claude/skills/hvac-designer/examples/riyadh_villa/output/out/HVAC_BOQ.xlsx
@@ -791,7 +791,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>DS-24: 7.0 kW nominal cooling, 380 L/s, ESP 75 Pa, heat 7.6 kW, R410A</t>
+          <t>DS-18: 5.3 kW nominal cooling, 300 L/s, ESP 75 Pa, heat 5.8 kW, R410A</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>DS-O-24: 7.0 kW nominal, 2.19 kW input, T3 rated, anti-vibration mounts</t>
+          <t>DS-O-18: 5.3 kW nominal, 1.66 kW input, T3 rated, anti-vibration mounts</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>6.15</v>
+        <v>4.12</v>
       </c>
       <c r="F23" s="7" t="n">
         <v>10</v>
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>23.81</v>
+        <v>24.81</v>
       </c>
       <c r="F24" s="7" t="n">
         <v>10</v>
@@ -1265,7 +1265,7 @@
         </is>
       </c>
       <c r="E25" s="6" t="n">
-        <v>15.25</v>
+        <v>14.83</v>
       </c>
       <c r="F25" s="7" t="n">
         <v>10</v>
@@ -1341,7 +1341,7 @@
         </is>
       </c>
       <c r="E27" s="6" t="n">
-        <v>15.1</v>
+        <v>10.32</v>
       </c>
       <c r="F27" s="7" t="n">
         <v>10</v>
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>13.95</v>
+        <v>18.07</v>
       </c>
       <c r="F28" s="7" t="n">
         <v>10</v>
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="E29" s="6" t="n">
-        <v>11.75</v>
+        <v>11.52</v>
       </c>
       <c r="F29" s="7" t="n">
         <v>10</v>
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>2.44</v>
+        <v>2.38</v>
       </c>
       <c r="F32" s="7" t="n">
         <v>10</v>
@@ -1508,7 +1508,7 @@
         </is>
       </c>
       <c r="E33" s="6" t="n">
-        <v>2.94</v>
+        <v>2.88</v>
       </c>
       <c r="F33" s="7" t="n">
         <v>10</v>
@@ -1584,7 +1584,7 @@
         </is>
       </c>
       <c r="E35" s="6" t="n">
-        <v>2.44</v>
+        <v>2.38</v>
       </c>
       <c r="F35" s="7" t="n">
         <v>10</v>
@@ -1622,7 +1622,7 @@
         </is>
       </c>
       <c r="E36" s="6" t="n">
-        <v>2.94</v>
+        <v>2.88</v>
       </c>
       <c r="F36" s="7" t="n">
         <v>10</v>
@@ -1759,7 +1759,7 @@
         </is>
       </c>
       <c r="E41" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F41" s="7" t="n">
         <v>0</v>
@@ -1775,7 +1775,7 @@
       </c>
       <c r="I41" s="6" t="inlineStr">
         <is>
-          <t>Tags: SD-FF-04, SD-FF-05, SD-FF-06, SD-FF-12</t>
+          <t>Tags: SD-FF-04, SD-FF-05, SD-FF-06</t>
         </is>
       </c>
     </row>
@@ -1843,7 +1843,7 @@
         </is>
       </c>
       <c r="E43" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F43" s="7" t="n">
         <v>0</v>
@@ -1859,7 +1859,7 @@
       </c>
       <c r="I43" s="6" t="inlineStr">
         <is>
-          <t>Tags: SD-FF-01, SD-FF-02</t>
+          <t>Tags: SD-FF-01, SD-FF-02, SD-FF-12</t>
         </is>
       </c>
     </row>
@@ -2689,7 +2689,7 @@
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>350x300</t>
+          <t>300x300</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
@@ -3448,7 +3448,7 @@
         </is>
       </c>
       <c r="E87" s="6" t="n">
-        <v>36.3</v>
+        <v>63.5</v>
       </c>
       <c r="F87" s="7" t="n">
         <v>10</v>
@@ -3490,7 +3490,7 @@
         </is>
       </c>
       <c r="E88" s="6" t="n">
-        <v>120.9</v>
+        <v>97.5</v>
       </c>
       <c r="F88" s="7" t="n">
         <v>10</v>
@@ -3532,7 +3532,7 @@
         </is>
       </c>
       <c r="E89" s="6" t="n">
-        <v>21.7</v>
+        <v>47</v>
       </c>
       <c r="F89" s="7" t="n">
         <v>10</v>
@@ -3574,7 +3574,7 @@
         </is>
       </c>
       <c r="E90" s="6" t="n">
-        <v>106.3</v>
+        <v>81</v>
       </c>
       <c r="F90" s="7" t="n">
         <v>10</v>
@@ -3616,7 +3616,7 @@
         </is>
       </c>
       <c r="E91" s="6" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F91" s="7" t="n">
         <v>10</v>
@@ -3654,7 +3654,7 @@
         </is>
       </c>
       <c r="E92" s="6" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="F92" s="7" t="n">
         <v>10</v>
@@ -3692,7 +3692,7 @@
         </is>
       </c>
       <c r="E93" s="6" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F93" s="7" t="n">
         <v>10</v>
@@ -3730,7 +3730,7 @@
         </is>
       </c>
       <c r="E94" s="6" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="F94" s="7" t="n">
         <v>10</v>
@@ -3783,7 +3783,7 @@
         </is>
       </c>
       <c r="E97" s="6" t="n">
-        <v>40.16</v>
+        <v>39</v>
       </c>
       <c r="F97" s="7" t="n">
         <v>10</v>
@@ -3821,7 +3821,7 @@
         </is>
       </c>
       <c r="E98" s="6" t="n">
-        <v>5.37</v>
+        <v>5.29</v>
       </c>
       <c r="F98" s="7" t="n">
         <v>10</v>
@@ -3859,7 +3859,7 @@
         </is>
       </c>
       <c r="E99" s="6" t="n">
-        <v>34.81</v>
+        <v>34.11</v>
       </c>
       <c r="F99" s="7" t="n">
         <v>10</v>
@@ -3935,7 +3935,7 @@
         </is>
       </c>
       <c r="E101" s="6" t="n">
-        <v>36.3</v>
+        <v>63.5</v>
       </c>
       <c r="F101" s="7" t="n">
         <v>10</v>
@@ -3973,7 +3973,7 @@
         </is>
       </c>
       <c r="E102" s="6" t="n">
-        <v>120.9</v>
+        <v>97.5</v>
       </c>
       <c r="F102" s="7" t="n">
         <v>10</v>
@@ -4011,7 +4011,7 @@
         </is>
       </c>
       <c r="E103" s="6" t="n">
-        <v>21.7</v>
+        <v>47</v>
       </c>
       <c r="F103" s="7" t="n">
         <v>10</v>
@@ -4049,7 +4049,7 @@
         </is>
       </c>
       <c r="E104" s="6" t="n">
-        <v>106.3</v>
+        <v>81</v>
       </c>
       <c r="F104" s="7" t="n">
         <v>10</v>
@@ -4102,7 +4102,7 @@
         </is>
       </c>
       <c r="E107" s="6" t="n">
-        <v>8.93</v>
+        <v>8.91</v>
       </c>
       <c r="F107" s="7" t="n">
         <v>10</v>
@@ -4182,7 +4182,7 @@
         </is>
       </c>
       <c r="E109" s="6" t="n">
-        <v>19.06</v>
+        <v>21.03</v>
       </c>
       <c r="F109" s="7" t="n">
         <v>10</v>
@@ -4315,7 +4315,7 @@
         </is>
       </c>
       <c r="E114" s="6" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F114" s="7" t="n">
         <v>5</v>
@@ -4353,7 +4353,7 @@
         </is>
       </c>
       <c r="E115" s="6" t="n">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F115" s="7" t="n">
         <v>5</v>
@@ -4391,7 +4391,7 @@
         </is>
       </c>
       <c r="E116" s="6" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F116" s="7" t="n">
         <v>5</v>

</xml_diff>